<commit_message>
feat(profile): add complete Profile API with 9 endpoints
- Implement GET/PATCH/DELETE /users/me, food-log CRUD, avatar upload, change-password, and food-log summary
- Add dedicated service layer (profile_service.py) and expanded schemas
- Add avatar_url column to Profile model; join user_preferences for enriched responses
- Update xlsx, API docs, .gitignore (uploads/), and .env.example with Supabase vars
- Include scan API modules and docs from prior work

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/required-api-document.xlsx
+++ b/required-api-document.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Backend" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -75,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -99,6 +99,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -377,19 +378,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" style="11" min="1" max="1"/>
+    <col width="16" customWidth="1" style="11" min="2" max="2"/>
+    <col width="24" customWidth="1" style="11" min="3" max="3"/>
+    <col width="22" customWidth="1" style="11" min="4" max="4"/>
+    <col width="52" customWidth="1" style="11" min="5" max="5"/>
+    <col width="10" customWidth="1" style="11" min="6" max="6"/>
+    <col width="12" customWidth="1" style="11" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1" s="11">
       <c r="B1" s="2" t="inlineStr">
         <is>
           <t>JWT 필요한 API는 Authorization: Bearer &lt;token&gt; 헤더 사용</t>
@@ -424,7 +425,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
+    <row r="2" ht="15.75" customHeight="1" s="11">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
@@ -440,7 +441,7 @@
       <c r="G2" s="2" t="n"/>
       <c r="I2" s="1" t="n"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
+    <row r="3" ht="15.75" customHeight="1" s="11">
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -462,7 +463,7 @@
       <c r="J3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" ht="15.75" customHeight="1" s="11">
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -491,7 +492,7 @@
       <c r="G4" s="3" t="n"/>
       <c r="J4" s="1" t="n"/>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
+    <row r="5" ht="15.75" customHeight="1" s="11">
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -521,7 +522,7 @@
       <c r="J5" s="1" t="n"/>
       <c r="L5" s="1" t="n"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" ht="15.75" customHeight="1" s="11">
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -549,7 +550,7 @@
       </c>
       <c r="G6" s="3" t="n"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" ht="15.75" customHeight="1" s="11">
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -577,7 +578,7 @@
       </c>
       <c r="G7" s="3" t="n"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="15.75" customHeight="1" s="11">
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -606,7 +607,7 @@
       </c>
       <c r="G8" s="3" t="n"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="15.75" customHeight="1" s="11">
       <c r="A9" s="1" t="n"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -635,7 +636,7 @@
       </c>
       <c r="G9" s="3" t="n"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="15.75" customHeight="1" s="11">
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -664,7 +665,7 @@
       </c>
       <c r="G10" s="3" t="n"/>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="15.75" customHeight="1" s="11">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -693,7 +694,7 @@
       </c>
       <c r="G11" s="3" t="n"/>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1" s="11">
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -722,7 +723,7 @@
       </c>
       <c r="G12" s="3" t="n"/>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" ht="15.75" customHeight="1" s="11">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>GET</t>
@@ -750,7 +751,7 @@
       </c>
       <c r="G13" s="3" t="n"/>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1" s="11">
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="3" t="n"/>
@@ -758,7 +759,7 @@
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" ht="15.75" customHeight="1" s="11">
       <c r="A15" t="n">
         <v>2</v>
       </c>
@@ -773,7 +774,7 @@
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" ht="15.75" customHeight="1" s="11">
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -785,7 +786,7 @@
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="15.75" customHeight="1" s="11">
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>POST</t>
@@ -809,7 +810,7 @@
       </c>
       <c r="G17" s="3" t="n"/>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" ht="15.75" customHeight="1" s="11">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -838,7 +839,7 @@
       </c>
       <c r="G18" s="3" t="n"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1" s="11">
       <c r="B19" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
@@ -866,7 +867,7 @@
       </c>
       <c r="G19" s="3" t="n"/>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1" s="11">
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -874,7 +875,7 @@
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1" s="11">
       <c r="A21" t="n">
         <v>3</v>
       </c>
@@ -889,7 +890,7 @@
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1" s="11">
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -901,7 +902,7 @@
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1" s="11">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -937,13 +938,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
-      <c r="J23" s="6" t="n"/>
-      <c r="K23" s="6" t="n"/>
-      <c r="L23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="11">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -979,13 +975,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="11">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>V</t>
@@ -1021,13 +1012,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="11">
       <c r="A26" s="9" t="inlineStr">
         <is>
           <t>V</t>
@@ -1063,13 +1049,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="11">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1101,13 +1082,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="11">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1143,13 +1119,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="11">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1185,13 +1156,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="6" t="n"/>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="11">
       <c r="A30" t="n">
         <v>4</v>
       </c>
@@ -1206,7 +1172,7 @@
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1" s="11">
       <c r="B31" s="3" t="n"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -1218,7 +1184,7 @@
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1" s="11">
       <c r="A32" s="9" t="inlineStr">
         <is>
           <t>V</t>
@@ -1250,13 +1216,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="11">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1292,13 +1253,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="11">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1334,13 +1290,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
+    </row>
+    <row r="35" ht="15.75" customHeight="1" s="11">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1376,13 +1327,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="6" t="n"/>
-      <c r="J35" s="6" t="n"/>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="11">
       <c r="A36" s="9" t="inlineStr">
         <is>
           <t>V</t>
@@ -1418,13 +1364,8 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="11">
       <c r="A37" t="n">
         <v>5</v>
       </c>
@@ -1439,7 +1380,7 @@
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1" s="11">
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="5" t="inlineStr">
         <is>
@@ -1451,7 +1392,7 @@
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1" s="11">
       <c r="B39" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -1475,7 +1416,7 @@
       </c>
       <c r="G39" s="3" t="n"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1" s="11">
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -1503,7 +1444,7 @@
       </c>
       <c r="G40" s="3" t="n"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1" s="11">
       <c r="B41" s="3" t="n"/>
       <c r="C41" s="3" t="n"/>
       <c r="D41" s="3" t="n"/>
@@ -1511,7 +1452,7 @@
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="n"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="15.75" customHeight="1" s="11">
       <c r="A42" s="1" t="n">
         <v>6</v>
       </c>
@@ -1526,7 +1467,7 @@
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="15.75" customHeight="1" s="11">
       <c r="B43" s="2" t="n"/>
       <c r="C43" s="5" t="inlineStr">
         <is>
@@ -1538,7 +1479,7 @@
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1" s="11">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1575,7 +1516,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1" s="11">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1612,7 +1553,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1" s="11">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1649,7 +1590,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="15.75" customHeight="1" s="11">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>V</t>
@@ -1686,7 +1627,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="15.75" customHeight="1" s="11">
       <c r="B48" s="3" t="n"/>
       <c r="C48" s="3" t="n"/>
       <c r="D48" s="3" t="n"/>
@@ -1694,162 +1635,520 @@
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" t="n">
+    <row r="49" ht="15.75" customHeight="1" s="11">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>/community/posts/:postId</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>/likes</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>게시글에 좋아요를 누릅니다.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="11">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>/community/posts/:postId</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>/likes</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>게시글 좋아요를 취소합니다.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="11">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>/community/posts/:postId</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>/replies</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>게시글에 댓글을 작성합니다.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="11">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>/community/replies/:replyId</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>/replies</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>대댓글(중첩 댓글)을 작성합니다.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="11">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>/community/replies/:replyId</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>/likes</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>댓글에 좋아요를 누릅니다.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="11">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>/community/replies/:replyId</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>/likes</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>댓글 좋아요를 취소합니다.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="11">
+      <c r="A55" t="n">
         <v>7</v>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Profile</t>
         </is>
       </c>
-      <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="3" t="n"/>
-      <c r="G49" s="3" t="n"/>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="B50" s="3" t="n"/>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>사용자 프로필과 개인 식사 기록을 조회/수정합니다.</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
-      <c r="G50" s="3" t="n"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>/users</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>/me</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>내 프로필 정보를 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="n"/>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>/users/me</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>/food-log</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>내 식사 기록 전체를 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="n"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>/users/me</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>/food-log</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>과거 식사 기록을 수동으로 추가합니다.</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="n"/>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>PATCH</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>/users</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>/me</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>내 프로필 정보를 수정합니다.</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="n"/>
-    </row>
-    <row r="55" ht="15.75" customHeight="1">
-      <c r="B55" s="3" t="n"/>
       <c r="C55" s="3" t="n"/>
       <c r="D55" s="3" t="n"/>
       <c r="E55" s="3" t="n"/>
       <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
     </row>
-    <row r="56" ht="13" customHeight="1">
+    <row r="56" ht="13" customHeight="1" s="11">
       <c r="B56" s="3" t="n"/>
-      <c r="C56" s="3" t="n"/>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>사용자 프로필과 개인 식사 기록을 조회/수정합니다.</t>
+        </is>
+      </c>
       <c r="D56" s="3" t="n"/>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
     </row>
+    <row r="57">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>/users</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>/me</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>내 프로필 정보를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>/users/me</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>/food-log</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>내 식사 기록 전체를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>/users/me</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>/food-log</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>과거 식사 기록을 수동으로 추가합니다.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>/users</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>/me</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>내 프로필 정보를 수정합니다.</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>/users</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>/me</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>사용자 계정을 영구 삭제합니다.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>/users/me</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>/avatar</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>프로필 사진을 업로드합니다.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>/users/me</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>/change-password</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>비밀번호를 변경합니다.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>/users/me/food-log</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>/:entryId</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>식사 기록 항목을 삭제합니다.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>/users/me/food-log</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>/summary</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>영양 요약 및 연속 기록 데이터를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="3" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(questionnaire): implement Questionnaire API with 3 endpoints
Add POST /questionnaire, GET /users/me/preferences, and
PATCH /users/me/preferences with unit conversion (ft/lb → cm/kg),
Mifflin-St Jeor nutrition calculation, favorite dining halls,
and comprehensive input validation. Update docs accordingly.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/required-api-document.xlsx
+++ b/required-api-document.xlsx
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +106,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1393,56 +1406,84 @@
       <c r="G38" s="3" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="11">
-      <c r="B39" s="2" t="inlineStr">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>/scan</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="13" t="inlineStr">
         <is>
           <t>음식 사진을 분석해 음식/영양 정보를 반환합니다.</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="n"/>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="n"/>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="12" t="n"/>
+      <c r="K39" s="12" t="n"/>
+      <c r="L39" s="12" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="11">
-      <c r="B40" s="2" t="inlineStr">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>/scan</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>/log</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>인식된 음식 및 영양 정보를 식사 로그에 저장합니다.</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="n"/>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="n"/>
+      <c r="I40" s="12" t="n"/>
+      <c r="J40" s="12" t="n"/>
+      <c r="K40" s="12" t="n"/>
+      <c r="L40" s="12" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="11">
       <c r="B41" s="3" t="n"/>
@@ -1636,226 +1677,256 @@
       <c r="G48" s="3" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="11">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>/community/posts/:postId</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>/likes</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>게시글에 좋아요를 누릅니다.</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H49" s="12" t="n"/>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="12" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="11">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>/community/posts/:postId</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>/likes</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="12" t="inlineStr">
         <is>
           <t>게시글 좋아요를 취소합니다.</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="n"/>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="12" t="n"/>
+      <c r="K50" s="12" t="n"/>
+      <c r="L50" s="12" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="11">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>/community/posts/:postId</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>/replies</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>게시글에 댓글을 작성합니다.</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H51" s="12" t="n"/>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="12" t="n"/>
+      <c r="K51" s="12" t="n"/>
+      <c r="L51" s="12" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="11">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr">
         <is>
           <t>/community/replies/:replyId</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>/replies</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="12" t="inlineStr">
         <is>
           <t>대댓글(중첩 댓글)을 작성합니다.</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="12" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="11">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>/community/replies/:replyId</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>/likes</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>댓글에 좋아요를 누릅니다.</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="n"/>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
+      <c r="K53" s="12" t="n"/>
+      <c r="L53" s="12" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="11">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>/community/replies/:replyId</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>/likes</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="12" t="inlineStr">
         <is>
           <t>댓글 좋아요를 취소합니다.</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H54" s="12" t="n"/>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="12" t="n"/>
+      <c r="K54" s="12" t="n"/>
+      <c r="L54" s="12" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="11">
       <c r="A55" t="n">
@@ -1885,251 +1956,382 @@
       <c r="G56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="3" t="inlineStr">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C57" s="14" t="inlineStr">
         <is>
           <t>/users</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>/me</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>내 프로필 정보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="n"/>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H57" s="12" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="12" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="3" t="inlineStr">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>/food-log</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>내 식사 기록 전체를 조회합니다.</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="n"/>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G58" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H58" s="12" t="n"/>
+      <c r="I58" s="12" t="n"/>
+      <c r="J58" s="12" t="n"/>
+      <c r="K58" s="12" t="n"/>
+      <c r="L58" s="12" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="3" t="inlineStr">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="14" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>/food-log</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t>과거 식사 기록을 수동으로 추가합니다.</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="n"/>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H59" s="12" t="n"/>
+      <c r="I59" s="12" t="n"/>
+      <c r="J59" s="12" t="n"/>
+      <c r="K59" s="12" t="n"/>
+      <c r="L59" s="12" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="3" t="inlineStr">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>/users</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>/me</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>내 프로필 정보를 수정합니다.</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="n"/>
+      <c r="F60" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="12" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" t="inlineStr">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>/users</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>/me</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>사용자 계정을 영구 삭제합니다.</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F61" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H61" s="12" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="n"/>
+      <c r="K61" s="12" t="n"/>
+      <c r="L61" s="12" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" t="inlineStr">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>/avatar</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>프로필 사진을 업로드합니다.</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H62" s="12" t="n"/>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="12" t="n"/>
+      <c r="K62" s="12" t="n"/>
+      <c r="L62" s="12" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" t="inlineStr">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>/change-password</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="12" t="inlineStr">
         <is>
           <t>비밀번호를 변경합니다.</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="n"/>
+      <c r="I63" s="12" t="n"/>
+      <c r="J63" s="12" t="n"/>
+      <c r="K63" s="12" t="n"/>
+      <c r="L63" s="12" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" t="inlineStr">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
         <is>
           <t>/users/me/food-log</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>/:entryId</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="12" t="inlineStr">
         <is>
           <t>식사 기록 항목을 삭제합니다.</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="12" t="n"/>
+      <c r="K64" s="12" t="n"/>
+      <c r="L64" s="12" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" t="inlineStr">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>/users/me/food-log</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>/summary</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="12" t="inlineStr">
         <is>
           <t>영양 요약 및 연속 기록 데이터를 조회합니다.</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="n"/>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="12" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="12" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="3" t="n"/>

</xml_diff>

<commit_message>
feat: authentication security hardening and api documentation add
</commit_message>
<xml_diff>
--- a/required-api-document.xlsx
+++ b/required-api-document.xlsx
@@ -391,7 +391,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="11" min="1" max="1"/>
@@ -444,7 +444,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>User Service (로그인/회원가입)</t>
+          <t>Authentication (Supabase)</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
@@ -458,7 +458,7 @@
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>회원가입, 로그인, 이메일 인증, 비밀번호 재설정, 토큰 갱신을 처리합니다.</t>
+          <t>Supabase Auth (클라이언트) + 백엔드 3 endpoints. 프론트엔드가 Supabase JS SDK로 인증 처리.</t>
         </is>
       </c>
       <c r="D3" s="3" t="n"/>
@@ -502,7 +502,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
       <c r="J4" s="1" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="11">
@@ -531,7 +535,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
       <c r="J5" s="1" t="n"/>
       <c r="L5" s="1" t="n"/>
     </row>
@@ -561,7 +569,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="11">
       <c r="B7" s="2" t="inlineStr">
@@ -589,7 +601,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="11">
       <c r="A8" s="1" t="n"/>
@@ -618,7 +634,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="11">
       <c r="A9" s="1" t="n"/>
@@ -647,7 +667,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="11">
       <c r="A10" s="1" t="n"/>
@@ -676,7 +700,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="11">
       <c r="A11" s="1" t="n"/>
@@ -705,10 +733,18 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="11">
-      <c r="A12" s="1" t="n"/>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>POST</t>
@@ -734,9 +770,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n"/>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="11">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>GET</t>
@@ -762,167 +807,193 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="11">
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>/auth</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>/profile</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>프로필 생성/업데이트 (Supabase 인증 후 동기화)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="11">
-      <c r="A15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Questionnaire</t>
-        </is>
-      </c>
+      <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="3" t="n"/>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="11">
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>온보딩 및 프로필 수정에 필요한 식습관/신체 정보를 관리합니다.</t>
-        </is>
-      </c>
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Questionnaire</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="11">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>온보딩 및 프로필 수정에 필요한 식습관/신체 정보를 관리합니다.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="11">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>/questionnaire</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>초기 선호 정보(신체정보/식단/알러지)를 저장합니다.</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" s="11">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="11">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>/preferences</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>내 선호 정보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="11">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="11">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>/preferences</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>내 선호 정보를 수정합니다.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" s="11">
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="11">
-      <c r="A21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Homescreen (홈화면)</t>
-        </is>
-      </c>
+      <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -930,53 +1001,31 @@
       <c r="G21" s="3" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="11">
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>홈 화면 추천/목표/메뉴 요약/식사 기록 기능을 제공합니다.</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n"/>
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Homescreen (홈화면)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="11">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>/recommendations</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>/combo</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>개인 선호 기반 추천 콤보를 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>홈 화면 추천/목표/메뉴 요약/식사 기록 기능을 제공합니다.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="11">
       <c r="A24" s="6" t="inlineStr">
@@ -989,56 +1038,56 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>/recommendations</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>/combo</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>개인 선호 기반 추천 콤보를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="11">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>/goals</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>/daily</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>오늘의 칼로리/영양소 목표 진행률을 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="11">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>/menus</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>/summary</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>식당별 추천 메뉴 요약을 조회합니다.</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -1058,57 +1107,61 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>/menus</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>/summary</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>식당별 추천 메뉴 요약을 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="11">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>/meals</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>/log</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>선택한 음식으로 식사 기록을 저장합니다.</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="11">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>/favorites</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>추천 콤보를 즐겨찾기에 저장합니다.</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -1130,7 +1183,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1138,14 +1191,10 @@
           <t>/favorites</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>/:favoriteId</t>
-        </is>
-      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>저장한 즐겨찾기 콤보를 제거합니다.</t>
+          <t>추천 콤보를 즐겨찾기에 저장합니다.</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -1167,119 +1216,119 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>/favorites</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>/:favoriteId</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>저장한 즐겨찾기 콤보를 제거합니다.</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="11">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>/recommendations</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>/addons</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>추가 추천 음식 및 빠른 추가 항목을 조회합니다.</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" s="11">
-      <c r="A30" t="n">
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="11">
+      <c r="A31" t="n">
         <v>4</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Dining Hall</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" s="11">
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>식당, 스테이션, 스테이션별 메뉴 조회 API입니다.</t>
-        </is>
-      </c>
+      <c r="C31" s="2" t="n"/>
       <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
+      <c r="E31" s="2" t="n"/>
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="11">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>식당, 스테이션, 스테이션별 메뉴 조회 API입니다.</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="11">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>/dining-halls</t>
         </is>
       </c>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>전체 다이닝홀 목록을 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" s="11">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>/dining-halls</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>/:hallId</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>특정 다이닝홀 상세 정보를 조회합니다.</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -1306,17 +1355,17 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>/dining-halls/:hallId</t>
+          <t>/dining-halls</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>/stations</t>
+          <t>/:hallId</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>해당 다이닝홀의 스테이션 목록을 조회합니다.</t>
+          <t>특정 다이닝홀 상세 정보를 조회합니다.</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -1336,138 +1385,137 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>/dining-halls/:hallId</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
+          <t>/stations</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>해당 다이닝홀의 스테이션 목록을 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" s="11">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>/dining-halls/:hallId</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
           <t>/menus</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>스테이션별 메뉴를 조회합니다.</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F36" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1" s="11">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" s="11">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>/dining-halls</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>/full</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>프론트엔드 화면용 통합 다이닝홀 데이터를 조회합니다.</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" s="11">
-      <c r="A37" t="n">
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="11">
+      <c r="A38" t="n">
         <v>5</v>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Scan</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" s="11">
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>사진 인식 기반 음식 분석 및 로그 저장 기능입니다.</t>
-        </is>
-      </c>
+      <c r="C38" s="2" t="n"/>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="11">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>/scan</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>음식 사진을 분석해 음식/영양 정보를 반환합니다.</t>
-        </is>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="H39" s="12" t="n"/>
-      <c r="I39" s="12" t="n"/>
-      <c r="J39" s="12" t="n"/>
-      <c r="K39" s="12" t="n"/>
-      <c r="L39" s="12" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>사진 인식 기반 음식 분석 및 로그 저장 기능입니다.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="11">
       <c r="A40" s="12" t="inlineStr">
@@ -1485,14 +1533,10 @@
           <t>/scan</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>/log</t>
-        </is>
-      </c>
+      <c r="D40" s="14" t="n"/>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>인식된 음식 및 영양 정보를 식사 로그에 저장합니다.</t>
+          <t>음식 사진을 분석해 음식/영양 정보를 반환합니다.</t>
         </is>
       </c>
       <c r="F40" s="14" t="inlineStr">
@@ -1512,22 +1556,49 @@
       <c r="L40" s="12" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="11">
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>/scan</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>/log</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>인식된 음식 및 영양 정보를 식사 로그에 저장합니다.</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="n"/>
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="12" t="n"/>
+      <c r="K41" s="12" t="n"/>
+      <c r="L41" s="12" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="11">
-      <c r="A42" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Community</t>
-        </is>
-      </c>
+      <c r="B42" s="3" t="n"/>
       <c r="C42" s="3" t="n"/>
       <c r="D42" s="3" t="n"/>
       <c r="E42" s="3" t="n"/>
@@ -1535,53 +1606,31 @@
       <c r="G42" s="3" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="11">
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>커뮤니티 게시글 조회/작성/상세/삭제 API입니다.</t>
-        </is>
-      </c>
+      <c r="A43" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n"/>
       <c r="D43" s="3" t="n"/>
-      <c r="E43" s="2" t="n"/>
+      <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="11">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>/community</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>/posts</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>커뮤니티 게시글 피드를 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>커뮤니티 게시글 조회/작성/상세/삭제 API입니다.</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="11">
       <c r="A45" s="6" t="inlineStr">
@@ -1591,7 +1640,7 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
@@ -1606,12 +1655,12 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티 게시글을 작성합니다.</t>
+          <t>커뮤니티 게시글 피드를 조회합니다.</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -1628,27 +1677,27 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>/community/posts</t>
+          <t>/community</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>/:postId</t>
+          <t>/posts</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>게시글 상세를 조회합니다.</t>
+          <t>커뮤니티 게시글을 작성합니다.</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -1663,86 +1712,81 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>/community/posts</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>/:postId</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>게시글 상세를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="11">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>/community/posts</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>/:postId</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>내가 작성한 게시글을 삭제합니다.</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1" s="11">
-      <c r="B48" s="3" t="n"/>
-      <c r="C48" s="3" t="n"/>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
-      <c r="F48" s="3" t="n"/>
-      <c r="G48" s="3" t="n"/>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="11">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>/community/posts/:postId</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="inlineStr">
-        <is>
-          <t>/likes</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>게시글에 좋아요를 누릅니다.</t>
-        </is>
-      </c>
-      <c r="F49" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G49" s="12" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="H49" s="12" t="n"/>
-      <c r="I49" s="12" t="n"/>
-      <c r="J49" s="12" t="n"/>
-      <c r="K49" s="12" t="n"/>
-      <c r="L49" s="12" t="n"/>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="11">
       <c r="A50" s="12" t="inlineStr">
@@ -1752,7 +1796,7 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
@@ -1767,7 +1811,7 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>게시글 좋아요를 취소합니다.</t>
+          <t>게시글에 좋아요를 누릅니다.</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
@@ -1794,7 +1838,7 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
@@ -1804,12 +1848,12 @@
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>/replies</t>
+          <t>/likes</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>게시글에 댓글을 작성합니다.</t>
+          <t>게시글 좋아요를 취소합니다.</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
@@ -1841,7 +1885,7 @@
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>/community/replies/:replyId</t>
+          <t>/community/posts/:postId</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -1851,7 +1895,7 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>대댓글(중첩 댓글)을 작성합니다.</t>
+          <t>게시글에 댓글을 작성합니다.</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
@@ -1888,12 +1932,12 @@
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>/likes</t>
+          <t>/replies</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>댓글에 좋아요를 누릅니다.</t>
+          <t>대댓글(중첩 댓글)을 작성합니다.</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
@@ -1920,7 +1964,7 @@
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
@@ -1935,7 +1979,7 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>댓글 좋아요를 취소합니다.</t>
+          <t>댓글에 좋아요를 누릅니다.</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
@@ -1955,73 +1999,73 @@
       <c r="L54" s="12" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="11">
-      <c r="A55" t="n">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>/community/replies/:replyId</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>/likes</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
+          <t>댓글 좋아요를 취소합니다.</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H55" s="12" t="n"/>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="12" t="n"/>
+      <c r="K55" s="12" t="n"/>
+      <c r="L55" s="12" t="n"/>
+    </row>
+    <row r="56" ht="13" customHeight="1" s="11">
+      <c r="A56" t="n">
         <v>7</v>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Profile</t>
         </is>
       </c>
-      <c r="C55" s="3" t="n"/>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="n"/>
-    </row>
-    <row r="56" ht="13" customHeight="1" s="11">
-      <c r="B56" s="3" t="n"/>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>사용자 프로필과 개인 식사 기록을 조회/수정합니다.</t>
-        </is>
-      </c>
+      <c r="C56" s="3" t="n"/>
       <c r="D56" s="3" t="n"/>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>/users</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>/me</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>내 프로필 정보를 조회합니다.</t>
-        </is>
-      </c>
-      <c r="F57" s="14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>Built</t>
-        </is>
-      </c>
-      <c r="H57" s="12" t="n"/>
-      <c r="I57" s="12" t="n"/>
-      <c r="J57" s="12" t="n"/>
-      <c r="K57" s="12" t="n"/>
-      <c r="L57" s="12" t="n"/>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>사용자 프로필과 개인 식사 기록을 조회/수정합니다.</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -2036,17 +2080,17 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>/users/me</t>
+          <t>/users</t>
         </is>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>/food-log</t>
+          <t>/me</t>
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>내 식사 기록 전체를 조회합니다.</t>
+          <t>내 프로필 정보를 조회합니다.</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
@@ -2073,7 +2117,7 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -2088,7 +2132,7 @@
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
-          <t>과거 식사 기록을 수동으로 추가합니다.</t>
+          <t>내 식사 기록 전체를 조회합니다.</t>
         </is>
       </c>
       <c r="F59" s="14" t="inlineStr">
@@ -2115,22 +2159,22 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>/users</t>
+          <t>/users/me</t>
         </is>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>/me</t>
+          <t>/food-log</t>
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>내 프로필 정보를 수정합니다.</t>
+          <t>과거 식사 기록을 수동으로 추가합니다.</t>
         </is>
       </c>
       <c r="F60" s="14" t="inlineStr">
@@ -2155,32 +2199,32 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>DELETE</t>
-        </is>
-      </c>
-      <c r="C61" s="12" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
         <is>
           <t>/users</t>
         </is>
       </c>
-      <c r="D61" s="12" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>/me</t>
         </is>
       </c>
-      <c r="E61" s="12" t="inlineStr">
-        <is>
-          <t>사용자 계정을 영구 삭제합니다.</t>
-        </is>
-      </c>
-      <c r="F61" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G61" s="12" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>내 프로필 정보를 수정합니다.</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -2199,22 +2243,22 @@
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>/users/me</t>
+          <t>/users</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>/avatar</t>
+          <t>/me</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>프로필 사진을 업로드합니다.</t>
+          <t>사용자 계정을 영구 삭제합니다.</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
@@ -2251,12 +2295,12 @@
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>/change-password</t>
+          <t>/avatar</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>비밀번호를 변경합니다.</t>
+          <t>프로필 사진을 업로드합니다.</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
@@ -2283,22 +2327,22 @@
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
         <is>
-          <t>/users/me/food-log</t>
+          <t>/users/me</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>/:entryId</t>
+          <t>/change-password</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
         <is>
-          <t>식사 기록 항목을 삭제합니다.</t>
+          <t>비밀번호를 변경합니다.</t>
         </is>
       </c>
       <c r="F64" s="12" t="inlineStr">
@@ -2325,7 +2369,7 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
@@ -2335,12 +2379,12 @@
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>/summary</t>
+          <t>/:entryId</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>영양 요약 및 연속 기록 데이터를 조회합니다.</t>
+          <t>식사 기록 항목을 삭제합니다.</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
@@ -2360,12 +2404,46 @@
       <c r="L65" s="12" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>/users/me/food-log</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>/summary</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>영양 요약 및 연속 기록 데이터를 조회합니다.</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="n"/>
+      <c r="I66" s="12" t="n"/>
+      <c r="J66" s="12" t="n"/>
+      <c r="K66" s="12" t="n"/>
+      <c r="L66" s="12" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="3" t="n"/>
@@ -2375,6 +2453,14 @@
       <c r="F67" s="3" t="n"/>
       <c r="G67" s="3" t="n"/>
     </row>
+    <row r="68">
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
fix(auth): replaced user_id dependencies to JWT token
</commit_message>
<xml_diff>
--- a/required-api-document.xlsx
+++ b/required-api-document.xlsx
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,18 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -81,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -112,6 +124,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -391,7 +423,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="11" min="1" max="1"/>
@@ -477,32 +509,37 @@
       <c r="L3" s="1" t="n"/>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="11">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>/signin</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>이메일/비밀번호 로그인 후 액세스 토큰을 반환합니다.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
@@ -510,32 +547,37 @@
       <c r="J4" s="1" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="11">
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>/signup</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>회원가입 후 이메일 인증 코드를 발송합니다.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
@@ -544,307 +586,333 @@
       <c r="L5" s="1" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="11">
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>/google</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>구글 ID 토큰으로 로그인/회원가입을 처리합니다.</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="11">
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>/forgot-pw</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>비밀번호 재설정을 위한 인증 코드를 발송합니다.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="11">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>/verify-email</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>6자리 인증 코드로 이메일 인증을 완료합니다.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="11">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>/resend-code</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>인증 코드를 재전송합니다.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="11">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>/reset-pw</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>이메일 인증 후 비밀번호를 변경합니다.</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="11">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>/refresh-token</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>리프레시 토큰으로 액세스 토큰을 재발급합니다.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="11">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>/logout</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>현재 세션을 로그아웃 처리합니다.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="11">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>/me</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>현재 로그인한 사용자 정보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="11">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>/auth</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>/profile</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>프로필 생성/업데이트 (Supabase 인증 후 동기화)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -886,107 +954,107 @@
       <c r="G17" s="3" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="11">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>/questionnaire</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>초기 선호 정보(신체정보/식단/알러지)를 저장합니다.</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="11">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>/preferences</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>내 선호 정보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="11">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>/users/me</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>/preferences</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>내 선호 정보를 수정합니다.</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1028,255 +1096,255 @@
       <c r="G23" s="3" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="11">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>/recommendations</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>/combo</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>개인 선호 기반 추천 콤보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="11">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>/goals</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>/daily</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t>오늘의 칼로리/영양소 목표 진행률을 조회합니다.</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="11">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>/menus</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>/summary</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>식당별 추천 메뉴 요약을 조회합니다.</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="11">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>/meals</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>/log</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>선택한 음식으로 식사 기록을 저장합니다.</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="11">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>/favorites</t>
         </is>
       </c>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>추천 콤보를 즐겨찾기에 저장합니다.</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="11">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>/favorites</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>/:favoriteId</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>저장한 즐겨찾기 콤보를 제거합니다.</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="11">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>/recommendations</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>/addons</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E30" s="13" t="inlineStr">
         <is>
           <t>추가 추천 음식 및 빠른 추가 항목을 조회합니다.</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1310,181 +1378,181 @@
       <c r="G32" s="3" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="11">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>/dining-halls</t>
         </is>
       </c>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>전체 다이닝홀 목록을 조회합니다.</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="11">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>/dining-halls</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>/:hallId</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="13" t="inlineStr">
         <is>
           <t>특정 다이닝홀 상세 정보를 조회합니다.</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G34" s="8" t="inlineStr">
+      <c r="G34" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="11">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>/dining-halls/:hallId</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>/stations</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="13" t="inlineStr">
         <is>
           <t>해당 다이닝홀의 스테이션 목록을 조회합니다.</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="11">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>/dining-halls/:hallId</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>/menus</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>스테이션별 메뉴를 조회합니다.</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr">
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="11">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
         <is>
           <t>/dining-halls</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>/full</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>프론트엔드 화면용 통합 다이닝홀 데이터를 조회합니다.</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G37" s="8" t="inlineStr">
+      <c r="G37" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1549,11 +1617,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H40" s="12" t="n"/>
-      <c r="I40" s="12" t="n"/>
-      <c r="J40" s="12" t="n"/>
-      <c r="K40" s="12" t="n"/>
-      <c r="L40" s="12" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="11">
       <c r="A41" s="12" t="inlineStr">
@@ -1591,11 +1654,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H41" s="12" t="n"/>
-      <c r="I41" s="12" t="n"/>
-      <c r="J41" s="12" t="n"/>
-      <c r="K41" s="12" t="n"/>
-      <c r="L41" s="12" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="11">
       <c r="B42" s="3" t="n"/>
@@ -1633,148 +1691,148 @@
       <c r="G44" s="3" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="11">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>/community</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>/posts</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>커뮤니티 게시글 피드를 조회합니다.</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G45" s="8" t="inlineStr">
+      <c r="G45" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="11">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>/community</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>/posts</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>커뮤니티 게시글을 작성합니다.</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="11">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>/community/posts</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>/:postId</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="13" t="inlineStr">
         <is>
           <t>게시글 상세를 조회합니다.</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
+      <c r="G47" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="11">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>/community/posts</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>/:postId</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>내가 작성한 게시글을 삭제합니다.</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
@@ -1824,11 +1882,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H50" s="12" t="n"/>
-      <c r="I50" s="12" t="n"/>
-      <c r="J50" s="12" t="n"/>
-      <c r="K50" s="12" t="n"/>
-      <c r="L50" s="12" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="11">
       <c r="A51" s="12" t="inlineStr">
@@ -1866,11 +1919,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H51" s="12" t="n"/>
-      <c r="I51" s="12" t="n"/>
-      <c r="J51" s="12" t="n"/>
-      <c r="K51" s="12" t="n"/>
-      <c r="L51" s="12" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="11">
       <c r="A52" s="12" t="inlineStr">
@@ -1908,11 +1956,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H52" s="12" t="n"/>
-      <c r="I52" s="12" t="n"/>
-      <c r="J52" s="12" t="n"/>
-      <c r="K52" s="12" t="n"/>
-      <c r="L52" s="12" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="11">
       <c r="A53" s="12" t="inlineStr">
@@ -1950,11 +1993,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H53" s="12" t="n"/>
-      <c r="I53" s="12" t="n"/>
-      <c r="J53" s="12" t="n"/>
-      <c r="K53" s="12" t="n"/>
-      <c r="L53" s="12" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="11">
       <c r="A54" s="12" t="inlineStr">
@@ -1992,11 +2030,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H54" s="12" t="n"/>
-      <c r="I54" s="12" t="n"/>
-      <c r="J54" s="12" t="n"/>
-      <c r="K54" s="12" t="n"/>
-      <c r="L54" s="12" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="11">
       <c r="A55" s="12" t="inlineStr">
@@ -2034,11 +2067,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H55" s="12" t="n"/>
-      <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="n"/>
-      <c r="K55" s="12" t="n"/>
-      <c r="L55" s="12" t="n"/>
     </row>
     <row r="56" ht="13" customHeight="1" s="11">
       <c r="A56" t="n">
@@ -2103,11 +2131,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H58" s="12" t="n"/>
-      <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="n"/>
-      <c r="K58" s="12" t="n"/>
-      <c r="L58" s="12" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
@@ -2145,11 +2168,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H59" s="12" t="n"/>
-      <c r="I59" s="12" t="n"/>
-      <c r="J59" s="12" t="n"/>
-      <c r="K59" s="12" t="n"/>
-      <c r="L59" s="12" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -2187,11 +2205,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H60" s="12" t="n"/>
-      <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="n"/>
-      <c r="K60" s="12" t="n"/>
-      <c r="L60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
@@ -2229,11 +2242,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H61" s="12" t="n"/>
-      <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="n"/>
-      <c r="K61" s="12" t="n"/>
-      <c r="L61" s="12" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
@@ -2271,11 +2279,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H62" s="12" t="n"/>
-      <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="n"/>
-      <c r="K62" s="12" t="n"/>
-      <c r="L62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
@@ -2313,11 +2316,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H63" s="12" t="n"/>
-      <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="n"/>
-      <c r="K63" s="12" t="n"/>
-      <c r="L63" s="12" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -2355,11 +2353,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H64" s="12" t="n"/>
-      <c r="I64" s="12" t="n"/>
-      <c r="J64" s="12" t="n"/>
-      <c r="K64" s="12" t="n"/>
-      <c r="L64" s="12" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
@@ -2397,11 +2390,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H65" s="12" t="n"/>
-      <c r="I65" s="12" t="n"/>
-      <c r="J65" s="12" t="n"/>
-      <c r="K65" s="12" t="n"/>
-      <c r="L65" s="12" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
@@ -2439,11 +2427,6 @@
           <t>Built</t>
         </is>
       </c>
-      <c r="H66" s="12" t="n"/>
-      <c r="I66" s="12" t="n"/>
-      <c r="J66" s="12" t="n"/>
-      <c r="K66" s="12" t="n"/>
-      <c r="L66" s="12" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="3" t="n"/>
@@ -2461,7 +2444,17 @@
       <c r="F68" s="3" t="n"/>
       <c r="G68" s="3" t="n"/>
     </row>
+    <row r="69">
+      <c r="B69" s="24" t="inlineStr">
+        <is>
+          <t>범례:  V = 완료 표시  |  녹색 = 백엔드에서 구현한 API  |  연청 = Supabase 인증(프론트 SDK, 설계·문서 반영 완료)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B69:G69"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>